<commit_message>
feat: implement comprehensive analysis pipeline and generate validation results, visualizations, and documentation tables.
</commit_message>
<xml_diff>
--- a/results/TFL/listados/listing1_discrepancias_detalladas.xlsx
+++ b/results/TFL/listados/listing1_discrepancias_detalladas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,128 +456,128 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gemma-4-31B-it (Local)</t>
+          <t>Gemma-4-31B-it</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Historia #45</t>
+          <t>Historia #14</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>b280, d850, e1101, e355, e570</t>
+          <t>b280, d230, d430, d450, d640</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>b280, d850, e1101, e355</t>
+          <t>b280, d230, d430, d450, d640</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>b280, d850, e1101, e355</t>
+          <t>b147, b280, d230, d430, d450, d640</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>b280, d850, e1101, e355</t>
+          <t>b280, d230, d430, d450, d640</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>e570</t>
+          <t>b147</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gemma-4-31B-it (Local)</t>
+          <t>Gemma-4-31B-it</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Historia #62</t>
+          <t>Historia #34</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e310, e410</t>
+          <t>b280, e410</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e310, e410</t>
+          <t>b280, e410</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e310, e355, e410</t>
+          <t>b280, e310, e410</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e310, e410</t>
+          <t>b280, e410</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>e355</t>
+          <t>e310</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+          <t>Gemma-4-31B-it</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Historia #19</t>
+          <t>Historia #59</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>b134, b280, e1101</t>
+          <t>b130, d240, d920, e410</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e355</t>
+          <t>b130, b152, d240, d920, e410</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>b134, b280, e1101</t>
+          <t>b130, d240, d920, e410</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>b134, b280, e1101</t>
+          <t>b130, d240, d920, e410</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>e355</t>
+          <t>b152</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+          <t>Gemma-4-31B-it</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Historia #62</t>
+          <t>Historia #61</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e310, e355, e410</t>
+          <t>b134, b280, e1101, e410</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -587,54 +587,794 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e310, e355, e410</t>
+          <t>b134, b280, e1101, e410</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>b134, b280, e1101, e310, e410</t>
+          <t>b134, b280, e1101, e410</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>e355</t>
+          <t>e310</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gemini Flash 3.6 (Cloud)</t>
+          <t>Gemma-4-31B-it</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Todas (114/114)</t>
+          <t>Historia #102</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Acuerdo perfecto</t>
+          <t>b147, b152, b280, b760, d450</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Acuerdo perfecto</t>
+          <t>b147, b280, b760, d450</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Acuerdo perfecto</t>
+          <t>b147, b152, b280, b760, d450</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>100% Determinista</t>
+          <t>b147, b280, b760, d450</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Ninguno (0 discrepancias)</t>
+          <t>b152</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gemma-4-31B-it</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Historia #104</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>b280, b730, b760, d450, d850</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>b280, b730, d450, d850</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>b280, b730, d450, d850</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>b280, b730, d450, d850</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>b760</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Gemma-4-31B-it</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Historia #111</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>b130, b280, b455, d450, e1101, e355</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>b130, b280, b455, d230, d450, e1101, e355</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>b130, b280, b455, d230, d450, e1101, e355</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>b130, b280, b455, d450, e1101, e355</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>d230</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Historia #5</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>b152, b1602, b280, d240, d850, e570</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>b130, b152, b1602, b280, d240, d850, e570</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>b130, b152, b1602, b280, d240, d850, e570</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>b152, b1602, b280, d240, d850, e570</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>b130</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Historia #7</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Historia #9</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Historia #51</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>b130, b147, b280</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>b130, b147, b280</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>b130, b147, b280, b455</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>b130, b147, b280</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>b455</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Historia #58</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>b130, d230, d240, d770, d920, e410</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>b130, d230, d240, d770, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>b130, d230, d240, d920, e410</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>b130, d230, d240, d920, e410</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>d770, e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Historia #63</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>b134, b280, d760, e1101, e310, e410</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>b134, b280, d760, e1101, e410</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>b134, b280, d760, e1101, e310, e410</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>b134, b280, d760, e1101, e410</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Historia #73</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, d770, e410</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, e410</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, d770, e410</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, e410</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>d770</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Historia #75</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, e410</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, d760, e410</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, d760, e310, e410</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>b147, b280, b730, b760, e410</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>d760, e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Historia #81</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>b1602, b280, d770, e1101, e355</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>b1602, b280, d770, e1101, e355</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>b152, b1602, b280, d770, e1101, e355</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>b1602, b280, d770, e1101, e355</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>b152</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Historia #88</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>b280, d175, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>b280, d175, d920, e410</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>b280, d175, d920, e410</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>b280, d175, d920, e410</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Historia #90</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>b152, b280, d175, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>b152, b280, d175, d920, e410</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>b152, b280, d175, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>b152, b280, d175, d920, e410</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.5 (Cloud - Línea Base)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Historia #105</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>b280, b730, d450, d850</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>b280, b730, b760, d450, d850</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>b280, b730, d450, d850</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>b280, b730, d450, d850</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>b760</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.7</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Historia #7</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.7</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Historia #9</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e310, e410</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>b134, b152, b280, d240, d640, d760, d920, e410</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.7</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Historia #34</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>b280, e410</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>b280, d770, e410</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>b280, d770, e410</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>b280, e410</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>d770</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.7</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Historia #62</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>b134, b280, e1101, e355, e410</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>b134, b280, e1101, e355, e410</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>b134, b280, e1101, e310, e355, e410</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>b134, b280, e1101, e355, e410</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>e310</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.7</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Historia #63</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>b134, b280, d760, e1101, e410</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>b134, b280, d760, e1101, e410</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>b134, b280, e1101, e410</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>b134, b280, e1101, e410</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>d760</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Gemini Flash 3.7</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Historia #102</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>b147, b280, b760, d450</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>b147, b152, b280, b760, d450</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>b147, b280, b760, d450</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>b147, b280, b760, d450</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>b152</t>
         </is>
       </c>
     </row>

</xml_diff>